<commit_message>
Actualiza información BD Mongo DB
</commit_message>
<xml_diff>
--- a/postgresql/schemaEcommify_olist_analytics/ER ModeloConceptual.xlsx
+++ b/postgresql/schemaEcommify_olist_analytics/ER ModeloConceptual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_REPOS\maestria\Ecommify_Database_Design\postgresql\schemaEcommify_olist_analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13CFDFB-A298-4197-B25B-87AD53E589F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608E4FE3-86C0-441C-A3F8-2AECDB0BCFE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Olist Optimizado" sheetId="1" r:id="rId1"/>
@@ -120,15 +120,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>762993</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>585631</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>86710</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>375454</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>183346</xdr:rowOff>
+      <xdr:colOff>196187</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>115751</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -151,8 +151,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="762993" y="1742661"/>
-          <a:ext cx="4820565" cy="5398076"/>
+          <a:off x="585631" y="2254469"/>
+          <a:ext cx="4813177" cy="5349903"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>